<commit_message>
Added final dashboard with correct variance %
</commit_message>
<xml_diff>
--- a/Dashboard/Financial_dashboard.xlsx
+++ b/Dashboard/Financial_dashboard.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f0292d34bed0d210/Documents/GitHub/amazon-finance-variance-analysis/Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="11_F25DC773A252ABDACC1048005118739A5ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F2F2AF54-898F-420C-B590-2B9C95100EDC}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="11_F25DC773A252ABDACC1048005118739A5ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61D68DA1-E0F2-49F1-AAC9-A2BFE80DD219}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="1884" yWindow="1884" windowWidth="17280" windowHeight="8880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Budget_vs_Actual" sheetId="1" r:id="rId1"/>
@@ -27,17 +27,73 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="17">
   <si>
     <t>Key Insight: Marketing 12.5% over budget in Mar due to Q1 campaign - Dive Deep required</t>
+  </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Budget</t>
+  </si>
+  <si>
+    <t>Actual</t>
+  </si>
+  <si>
+    <t>Variance</t>
+  </si>
+  <si>
+    <t>Variance_%</t>
+  </si>
+  <si>
+    <t>Jan</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>Opertaions</t>
+  </si>
+  <si>
+    <t>Shipping</t>
+  </si>
+  <si>
+    <t>Technology</t>
+  </si>
+  <si>
+    <t>Feb</t>
+  </si>
+  <si>
+    <t>Mar</t>
+  </si>
+  <si>
+    <t>Apr</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>June</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -65,13 +121,37 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -82,6 +162,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -347,9 +431,521 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="6" max="6" width="10.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2">
+        <v>40000</v>
+      </c>
+      <c r="D2">
+        <v>45000</v>
+      </c>
+      <c r="E2">
+        <v>5000</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3">
+        <v>30000</v>
+      </c>
+      <c r="D3">
+        <v>28000</v>
+      </c>
+      <c r="E3">
+        <v>-2000</v>
+      </c>
+      <c r="F3" s="1">
+        <v>-6.7000000000000004E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4">
+        <v>25000</v>
+      </c>
+      <c r="D4">
+        <v>26500</v>
+      </c>
+      <c r="E4">
+        <v>1500</v>
+      </c>
+      <c r="F4" s="1">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5">
+        <v>35000</v>
+      </c>
+      <c r="D5">
+        <v>34500</v>
+      </c>
+      <c r="E5">
+        <v>-500</v>
+      </c>
+      <c r="F5" s="1">
+        <v>-1.4E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>40000</v>
+      </c>
+      <c r="D6">
+        <v>42000</v>
+      </c>
+      <c r="E6">
+        <v>2000</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7">
+        <v>30000</v>
+      </c>
+      <c r="D7">
+        <v>31000</v>
+      </c>
+      <c r="E7">
+        <v>1000</v>
+      </c>
+      <c r="F7" s="1">
+        <v>3.3000000000000002E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8">
+        <v>25000</v>
+      </c>
+      <c r="D8">
+        <v>24000</v>
+      </c>
+      <c r="E8">
+        <v>-1000</v>
+      </c>
+      <c r="F8" s="1">
+        <v>-0.04</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9">
+        <v>35000</v>
+      </c>
+      <c r="D9">
+        <v>38000</v>
+      </c>
+      <c r="E9">
+        <v>3000</v>
+      </c>
+      <c r="F9" s="1">
+        <v>8.5999999999999993E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10">
+        <v>45000</v>
+      </c>
+      <c r="D10">
+        <v>50625</v>
+      </c>
+      <c r="E10">
+        <v>5625</v>
+      </c>
+      <c r="F10" s="1">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11">
+        <v>30000</v>
+      </c>
+      <c r="D11">
+        <v>27500</v>
+      </c>
+      <c r="E11">
+        <v>-2500</v>
+      </c>
+      <c r="F11" s="1">
+        <v>-8.3000000000000004E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12">
+        <v>27000</v>
+      </c>
+      <c r="D12">
+        <v>29000</v>
+      </c>
+      <c r="E12">
+        <v>2000</v>
+      </c>
+      <c r="F12" s="1">
+        <v>7.3999999999999996E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13">
+        <v>35000</v>
+      </c>
+      <c r="D13">
+        <v>36000</v>
+      </c>
+      <c r="E13">
+        <v>1000</v>
+      </c>
+      <c r="F13" s="1">
+        <v>2.9000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14">
+        <v>40000</v>
+      </c>
+      <c r="D14">
+        <v>39500</v>
+      </c>
+      <c r="E14">
+        <v>-500</v>
+      </c>
+      <c r="F14" s="1">
+        <v>-1.2999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15">
+        <v>32000</v>
+      </c>
+      <c r="D15">
+        <v>30000</v>
+      </c>
+      <c r="E15">
+        <v>-2000</v>
+      </c>
+      <c r="F15" s="1">
+        <v>-6.3E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16">
+        <v>25000</v>
+      </c>
+      <c r="D16">
+        <v>25500</v>
+      </c>
+      <c r="E16">
+        <v>500</v>
+      </c>
+      <c r="F16" s="1">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17">
+        <v>40000</v>
+      </c>
+      <c r="D17">
+        <v>41000</v>
+      </c>
+      <c r="E17">
+        <v>1000</v>
+      </c>
+      <c r="F17" s="1">
+        <v>2.5000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18">
+        <v>42000</v>
+      </c>
+      <c r="D18">
+        <v>46000</v>
+      </c>
+      <c r="E18">
+        <v>4000</v>
+      </c>
+      <c r="F18" s="1">
+        <v>9.5000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19">
+        <v>30000</v>
+      </c>
+      <c r="D19">
+        <v>29500</v>
+      </c>
+      <c r="E19">
+        <v>-500</v>
+      </c>
+      <c r="F19" s="1">
+        <v>-1.7000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>15</v>
+      </c>
+      <c r="B20" t="s">
+        <v>10</v>
+      </c>
+      <c r="C20">
+        <v>26000</v>
+      </c>
+      <c r="D20">
+        <v>25000</v>
+      </c>
+      <c r="E20">
+        <v>-1000</v>
+      </c>
+      <c r="F20" s="1">
+        <v>-3.7999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>15</v>
+      </c>
+      <c r="B21" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21">
+        <v>35000</v>
+      </c>
+      <c r="D21">
+        <v>33000</v>
+      </c>
+      <c r="E21">
+        <v>-2000</v>
+      </c>
+      <c r="F21" s="1">
+        <v>-5.7000000000000002E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>16</v>
+      </c>
+      <c r="B22" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22">
+        <v>40000</v>
+      </c>
+      <c r="D22">
+        <v>43000</v>
+      </c>
+      <c r="E22">
+        <v>3000</v>
+      </c>
+      <c r="F22" s="1">
+        <v>7.4999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>16</v>
+      </c>
+      <c r="B23" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23">
+        <v>30000</v>
+      </c>
+      <c r="D23">
+        <v>28500</v>
+      </c>
+      <c r="E23">
+        <v>-1500</v>
+      </c>
+      <c r="F23" s="1">
+        <v>-0.05</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>16</v>
+      </c>
+      <c r="B24" t="s">
+        <v>10</v>
+      </c>
+      <c r="C24">
+        <v>25000</v>
+      </c>
+      <c r="D24">
+        <v>27000</v>
+      </c>
+      <c r="E24">
+        <v>2000</v>
+      </c>
+      <c r="F24" s="1">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>16</v>
+      </c>
+      <c r="B25" t="s">
+        <v>11</v>
+      </c>
+      <c r="C25">
+        <v>38000</v>
+      </c>
+      <c r="D25">
+        <v>39500</v>
+      </c>
+      <c r="E25">
+        <v>1500</v>
+      </c>
+      <c r="F25" s="1">
+        <v>3.9E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="F2:F25">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
+      <formula>0.021</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
+      <formula>0.021</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fixed Monthly_Trend with SUMIF totals - Mar 4.5% peak variance
</commit_message>
<xml_diff>
--- a/Dashboard/Financial_dashboard.xlsx
+++ b/Dashboard/Financial_dashboard.xlsx
@@ -5,29 +5,41 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f0292d34bed0d210/Documents/GitHub/amazon-finance-variance-analysis/Dashboard/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f0292d34bed0d210/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="11_F25DC773A252ABDACC1048005118739A5ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61D68DA1-E0F2-49F1-AAC9-A2BFE80DD219}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DA50B3B8-FC1C-4201-95E0-70C3EC025CB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Budget_vs_Actual" sheetId="1" r:id="rId1"/>
-    <sheet name="Summary_Pivot" sheetId="2" r:id="rId2"/>
-    <sheet name="Dashboard" sheetId="3" r:id="rId3"/>
+    <sheet name="Monthly_Trend" sheetId="2" r:id="rId2"/>
+    <sheet name="Executive_Summary" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="20">
   <si>
     <t>Key Insight: Marketing 12.5% over budget in Mar due to Q1 campaign - Dive Deep required</t>
   </si>
@@ -78,13 +90,26 @@
   </si>
   <si>
     <t>June</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   </t>
+  </si>
+  <si>
+    <t>Budget_Total</t>
+  </si>
+  <si>
+    <t>Actual_Total</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="44" formatCode="_-&quot;R&quot;* #,##0.00_-;\-&quot;R&quot;* #,##0.00_-;_-&quot;R&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="168" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -99,6 +124,19 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF222222"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -118,18 +156,23 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill>
@@ -141,13 +184,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -434,6 +470,7 @@
   <dimension ref="A1:F25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -939,10 +976,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F25">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
       <formula>0.021</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
       <formula>0.021</formula>
     </cfRule>
   </conditionalFormatting>
@@ -952,16 +989,139 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7FEBA24-B870-49E4-A59B-3C49DF4B6DC8}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.21875" customWidth="1"/>
+    <col min="4" max="4" width="10.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="3">
+        <f>SUMIF(Budget_vs_Actual!A:A,A2,Budget_vs_Actual!C:C)</f>
+        <v>130000</v>
+      </c>
+      <c r="C2" s="3">
+        <f>SUMIF(Budget_vs_Actual!A:A,A2,Budget_vs_Actual!D:D)</f>
+        <v>134000</v>
+      </c>
+      <c r="D2" s="5">
+        <f>(C2-B2)/B2</f>
+        <v>3.0769230769230771E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="3">
+        <f>SUMIF(Budget_vs_Actual!A:A,A3,Budget_vs_Actual!C:C)</f>
+        <v>130000</v>
+      </c>
+      <c r="C3" s="3">
+        <f>SUMIF(Budget_vs_Actual!A:A,A3,Budget_vs_Actual!D:D)</f>
+        <v>135000</v>
+      </c>
+      <c r="D3" s="5">
+        <f t="shared" ref="D3:D7" si="0">(C3-B3)/B3</f>
+        <v>3.8461538461538464E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="3">
+        <f>SUMIF(Budget_vs_Actual!A:A,A4,Budget_vs_Actual!C:C)</f>
+        <v>137000</v>
+      </c>
+      <c r="C4" s="3">
+        <f>SUMIF(Budget_vs_Actual!A:A,A4,Budget_vs_Actual!D:D)</f>
+        <v>143125</v>
+      </c>
+      <c r="D4" s="5">
+        <f t="shared" si="0"/>
+        <v>4.4708029197080293E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="3">
+        <f>SUMIF(Budget_vs_Actual!A:A,A5,Budget_vs_Actual!C:C)</f>
+        <v>137000</v>
+      </c>
+      <c r="C5" s="3">
+        <f>SUMIF(Budget_vs_Actual!A:A,A5,Budget_vs_Actual!D:D)</f>
+        <v>136000</v>
+      </c>
+      <c r="D5" s="5">
+        <f t="shared" si="0"/>
+        <v>-7.2992700729927005E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="3">
+        <f>SUMIF(Budget_vs_Actual!A:A,A6,Budget_vs_Actual!C:C)</f>
+        <v>133000</v>
+      </c>
+      <c r="C6" s="3">
+        <f>SUMIF(Budget_vs_Actual!A:A,A6,Budget_vs_Actual!D:D)</f>
+        <v>133500</v>
+      </c>
+      <c r="D6" s="5">
+        <f t="shared" si="0"/>
+        <v>3.7593984962406013E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="3">
+        <f>SUMIF(Budget_vs_Actual!A:A,A7,Budget_vs_Actual!C:C)</f>
+        <v>133000</v>
+      </c>
+      <c r="C7" s="3">
+        <f>SUMIF(Budget_vs_Actual!A:A,A7,Budget_vs_Actual!D:D)</f>
+        <v>138000</v>
+      </c>
+      <c r="D7" s="5">
+        <f t="shared" si="0"/>
+        <v>3.7593984962406013E-2</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5977D6E0-B54E-4E77-9658-8C63CC93E355}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
@@ -969,6 +1129,11 @@
         <v>0</v>
       </c>
     </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added Executive Summary with key insight - mar 4.5% / marketing 12.5%
</commit_message>
<xml_diff>
--- a/Dashboard/Financial_dashboard.xlsx
+++ b/Dashboard/Financial_dashboard.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f0292d34bed0d210/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f0292d34bed0d210/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DA50B3B8-FC1C-4201-95E0-70C3EC025CB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{56222C70-AA06-45E3-9D7D-4346B56F0E56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Budget_vs_Actual" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,6 @@
     <sheet name="Executive_Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,10 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="20">
-  <si>
-    <t>Key Insight: Marketing 12.5% over budget in Mar due to Q1 campaign - Dive Deep required</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="19">
   <si>
     <t>Month</t>
   </si>
@@ -92,13 +88,13 @@
     <t>June</t>
   </si>
   <si>
-    <t xml:space="preserve">   </t>
-  </si>
-  <si>
     <t>Budget_Total</t>
   </si>
   <si>
     <t>Actual_Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Key Insight: March peak variance 4,5% over budget  driven by Marketing +12,5% Q1 campaign. Other categories under budget offset it. April shows correction -0,7% due to cost control. </t>
   </si>
 </sst>
 </file>
@@ -107,7 +103,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="44" formatCode="_-&quot;R&quot;* #,##0.00_-;\-&quot;R&quot;* #,##0.00_-;_-&quot;R&quot;* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="168" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -165,8 +161,8 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -200,8 +196,1053 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-ZA"/>
+              <a:t>Budget</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-ZA" baseline="0"/>
+              <a:t> vs Actual Trend - Mar peak 4,5% variance</a:t>
+            </a:r>
+          </a:p>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:endParaRPr lang="en-ZA"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Monthly_Trend!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Budget_Total</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Monthly_Trend!$A$2:$A$7</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Jan</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>June</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Monthly_Trend!$B$2:$B$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>130000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>130000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>137000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>137000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>133000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>133000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-AA60-492C-ACB8-E10C470A6E2B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Monthly_Trend!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Actual_Total</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Monthly_Trend!$A$2:$A$7</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Jan</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>June</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Monthly_Trend!$C$2:$C$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>134000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>135000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>143125</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>136000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>133500</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>138000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-AA60-492C-ACB8-E10C470A6E2B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="1319865872"/>
+        <c:axId val="1120755408"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1319865872"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1120755408"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1120755408"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1319865872"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>45720</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>80010</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8E620DD4-302B-54C2-A148-EEF6269BF0CD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -476,30 +1517,30 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
         <v>7</v>
-      </c>
-      <c r="B2" t="s">
-        <v>8</v>
       </c>
       <c r="C2">
         <v>40000</v>
@@ -516,10 +1557,10 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C3">
         <v>30000</v>
@@ -536,10 +1577,10 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C4">
         <v>25000</v>
@@ -556,10 +1597,10 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C5">
         <v>35000</v>
@@ -576,10 +1617,10 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C6">
         <v>40000</v>
@@ -596,10 +1637,10 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C7">
         <v>30000</v>
@@ -616,10 +1657,10 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C8">
         <v>25000</v>
@@ -636,10 +1677,10 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C9">
         <v>35000</v>
@@ -656,10 +1697,10 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C10">
         <v>45000</v>
@@ -676,10 +1717,10 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C11">
         <v>30000</v>
@@ -696,10 +1737,10 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C12">
         <v>27000</v>
@@ -716,10 +1757,10 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C13">
         <v>35000</v>
@@ -736,10 +1777,10 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C14">
         <v>40000</v>
@@ -756,10 +1797,10 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C15">
         <v>32000</v>
@@ -776,10 +1817,10 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C16">
         <v>25000</v>
@@ -796,10 +1837,10 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C17">
         <v>40000</v>
@@ -816,10 +1857,10 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B18" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C18">
         <v>42000</v>
@@ -836,10 +1877,10 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B19" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C19">
         <v>30000</v>
@@ -856,10 +1897,10 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B20" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C20">
         <v>26000</v>
@@ -876,10 +1917,10 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B21" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C21">
         <v>35000</v>
@@ -896,10 +1937,10 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B22" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C22">
         <v>40000</v>
@@ -916,10 +1957,10 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B23" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C23">
         <v>30000</v>
@@ -936,10 +1977,10 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B24" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C24">
         <v>25000</v>
@@ -956,10 +1997,10 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B25" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C25">
         <v>38000</v>
@@ -999,21 +2040,21 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B2" s="3">
         <f>SUMIF(Budget_vs_Actual!A:A,A2,Budget_vs_Actual!C:C)</f>
@@ -1030,7 +2071,7 @@
     </row>
     <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3" s="3">
         <f>SUMIF(Budget_vs_Actual!A:A,A3,Budget_vs_Actual!C:C)</f>
@@ -1047,7 +2088,7 @@
     </row>
     <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" s="3">
         <f>SUMIF(Budget_vs_Actual!A:A,A4,Budget_vs_Actual!C:C)</f>
@@ -1064,7 +2105,7 @@
     </row>
     <row r="5" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" s="3">
         <f>SUMIF(Budget_vs_Actual!A:A,A5,Budget_vs_Actual!C:C)</f>
@@ -1081,7 +2122,7 @@
     </row>
     <row r="6" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B6" s="3">
         <f>SUMIF(Budget_vs_Actual!A:A,A6,Budget_vs_Actual!C:C)</f>
@@ -1098,7 +2139,7 @@
     </row>
     <row r="7" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B7" s="3">
         <f>SUMIF(Budget_vs_Actual!A:A,A7,Budget_vs_Actual!C:C)</f>
@@ -1121,20 +2162,43 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5977D6E0-B54E-4E77-9658-8C63CC93E355}">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="12.77734375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>17</v>
-      </c>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+    </row>
+    <row r="5" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+    </row>
+    <row r="6" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+    </row>
+    <row r="7" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+    </row>
+    <row r="8" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+    </row>
+    <row r="9" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>